<commit_message>
Regenerate files with Back to Top button
</commit_message>
<xml_diff>
--- a/starred_repos.xlsx
+++ b/starred_repos.xlsx
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>441444</v>
+        <v>441452</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -521,7 +521,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>22-11-2025 04:12</t>
+          <t>22-11-2025 04:36</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -557,11 +557,11 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>416613</v>
+        <v>416617</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>22-11-2025 04:13</t>
+          <t>22-11-2025 04:37</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>379995</v>
+        <v>380000</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -606,7 +606,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>22-11-2025 04:06</t>
+          <t>22-11-2025 04:34</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>270460</v>
+        <v>270463</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>22-11-2025 04:07</t>
+          <t>22-11-2025 04:36</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -687,11 +687,11 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>259310</v>
+        <v>259313</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>22-11-2025 03:55</t>
+          <t>22-11-2025 04:30</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -727,11 +727,11 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>250559</v>
+        <v>250560</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>22-11-2025 04:06</t>
+          <t>22-11-2025 04:37</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>198028</v>
+        <v>198029</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -776,7 +776,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>22-11-2025 04:13</t>
+          <t>22-11-2025 04:38</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -812,11 +812,11 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>195122</v>
+        <v>195125</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>22-11-2025 03:55</t>
+          <t>22-11-2025 04:37</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -852,7 +852,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>182891</v>
+        <v>182892</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -861,7 +861,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>22-11-2025 02:20</t>
+          <t>22-11-2025 04:30</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>157869</v>
+        <v>157872</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -906,7 +906,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>22-11-2025 04:07</t>
+          <t>22-11-2025 04:31</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>157014</v>
+        <v>157019</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -951,7 +951,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>22-11-2025 04:16</t>
+          <t>22-11-2025 04:33</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1032,7 +1032,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>135875</v>
+        <v>135876</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>22-11-2025 04:15</t>
+          <t>22-11-2025 04:20</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>115894</v>
+        <v>115895</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>22-11-2025 03:49</t>
+          <t>22-11-2025 04:20</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>115451</v>
+        <v>115454</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>22-11-2025 04:11</t>
+          <t>22-11-2025 04:35</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1297,7 +1297,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>102870</v>
+        <v>102871</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1306,7 +1306,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>22-11-2025 03:22</t>
+          <t>22-11-2025 04:36</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1342,7 +1342,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>102439</v>
+        <v>102443</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>22-11-2025 04:06</t>
+          <t>22-11-2025 04:37</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>93785</v>
+        <v>93786</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>22-11-2025 04:04</t>
+          <t>22-11-2025 04:28</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>92145</v>
+        <v>92146</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>22-11-2025 02:48</t>
+          <t>22-11-2025 04:35</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1562,11 +1562,11 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>88185</v>
+        <v>88187</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>22-11-2025 01:30</t>
+          <t>22-11-2025 04:38</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1647,7 +1647,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>84713</v>
+        <v>84714</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>22-11-2025 04:04</t>
+          <t>22-11-2025 04:29</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1692,7 +1692,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>83950</v>
+        <v>83955</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>22-11-2025 04:14</t>
+          <t>22-11-2025 04:31</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>83196</v>
+        <v>83197</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>22-11-2025 03:57</t>
+          <t>22-11-2025 04:21</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1867,7 +1867,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>78751</v>
+        <v>78752</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>22-11-2025 04:14</t>
+          <t>22-11-2025 04:33</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>75897</v>
+        <v>75898</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>22-11-2025 04:08</t>
+          <t>22-11-2025 04:20</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2002,7 +2002,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>70465</v>
+        <v>70466</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>22-11-2025 03:15</t>
+          <t>22-11-2025 04:38</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>68287</v>
+        <v>68291</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2056,7 +2056,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>22-11-2025 03:50</t>
+          <t>22-11-2025 04:32</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>67932</v>
+        <v>67933</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>22-11-2025 03:20</t>
+          <t>22-11-2025 04:23</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2137,11 +2137,11 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>66813</v>
+        <v>66814</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>22-11-2025 03:22</t>
+          <t>22-11-2025 04:23</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2307,7 +2307,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>58961</v>
+        <v>58962</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>22-11-2025 04:05</t>
+          <t>22-11-2025 04:25</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2523,11 +2523,11 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>53610</v>
+        <v>53611</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>22-11-2025 02:22</t>
+          <t>22-11-2025 04:31</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2698,7 +2698,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>51324</v>
+        <v>51325</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>22-11-2025 04:12</t>
+          <t>22-11-2025 04:26</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2788,7 +2788,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>47893</v>
+        <v>47892</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>22-11-2025 02:10</t>
+          <t>22-11-2025 04:23</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2874,7 +2874,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>47565</v>
+        <v>47566</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>22-11-2025 03:54</t>
+          <t>22-11-2025 04:30</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -3044,7 +3044,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -3053,7 +3053,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>22-11-2025 03:50</t>
+          <t>22-11-2025 04:38</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -3129,7 +3129,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>43207</v>
+        <v>43209</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>22-11-2025 04:09</t>
+          <t>22-11-2025 04:20</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3170,7 +3170,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>43133</v>
+        <v>43134</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -3179,7 +3179,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>22-11-2025 03:58</t>
+          <t>22-11-2025 04:21</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3215,7 +3215,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>42968</v>
+        <v>42969</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -3224,7 +3224,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>22-11-2025 03:35</t>
+          <t>22-11-2025 04:22</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3301,11 +3301,11 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>40991</v>
+        <v>40992</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>22-11-2025 03:36</t>
+          <t>22-11-2025 04:32</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3476,7 +3476,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>38977</v>
+        <v>38978</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -3485,7 +3485,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>22-11-2025 03:20</t>
+          <t>22-11-2025 04:32</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3656,7 +3656,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>36934</v>
+        <v>36935</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>22-11-2025 03:39</t>
+          <t>22-11-2025 04:26</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3921,7 +3921,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>34231</v>
+        <v>34232</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -3930,7 +3930,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>22-11-2025 03:54</t>
+          <t>22-11-2025 04:36</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -4092,7 +4092,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>31852</v>
+        <v>31853</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -4101,7 +4101,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>22-11-2025 03:31</t>
+          <t>22-11-2025 04:36</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -4262,7 +4262,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>31441</v>
+        <v>31442</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -4271,7 +4271,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>22-11-2025 04:06</t>
+          <t>22-11-2025 04:32</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -4352,7 +4352,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>29825</v>
+        <v>29826</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -4361,7 +4361,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>21-11-2025 23:19</t>
+          <t>22-11-2025 04:35</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -4487,11 +4487,11 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>28463</v>
+        <v>28464</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>21-11-2025 23:02</t>
+          <t>22-11-2025 04:33</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -4572,7 +4572,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>28093</v>
+        <v>28094</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -4581,7 +4581,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>22-11-2025 03:47</t>
+          <t>22-11-2025 04:38</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -4747,7 +4747,7 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>26858</v>
+        <v>26860</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -4756,7 +4756,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>22-11-2025 01:15</t>
+          <t>22-11-2025 04:35</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -5049,7 +5049,7 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>25587</v>
+        <v>25588</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -5058,7 +5058,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>22-11-2025 04:12</t>
+          <t>22-11-2025 04:21</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -5530,7 +5530,7 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>22126</v>
+        <v>22127</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -5539,7 +5539,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>22-11-2025 04:17</t>
+          <t>22-11-2025 04:35</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -5702,7 +5702,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>21404</v>
+        <v>21405</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
@@ -5711,7 +5711,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>22-11-2025 03:27</t>
+          <t>22-11-2025 04:35</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -5747,7 +5747,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>21059</v>
+        <v>21060</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -5756,7 +5756,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>21-11-2025 16:43</t>
+          <t>22-11-2025 04:28</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -5792,7 +5792,7 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>20685</v>
+        <v>20686</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
@@ -5801,7 +5801,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>22-11-2025 03:41</t>
+          <t>22-11-2025 04:35</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -5882,7 +5882,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>20583</v>
+        <v>20584</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>21-11-2025 22:21</t>
+          <t>22-11-2025 04:18</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -6151,7 +6151,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>22-11-2025 04:14</t>
+          <t>22-11-2025 04:18</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -6196,7 +6196,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>21-11-2025 19:42</t>
+          <t>22-11-2025 04:34</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -6457,7 +6457,7 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>17631</v>
+        <v>17632</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
@@ -6466,7 +6466,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>22-11-2025 02:33</t>
+          <t>22-11-2025 04:28</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -6767,7 +6767,7 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>16329</v>
+        <v>16330</v>
       </c>
       <c r="F145" t="inlineStr">
         <is>
@@ -6776,7 +6776,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>22-11-2025 03:18</t>
+          <t>22-11-2025 04:19</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
@@ -7073,7 +7073,7 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>15662</v>
+        <v>15663</v>
       </c>
       <c r="F152" t="inlineStr">
         <is>
@@ -7082,7 +7082,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>22-11-2025 04:00</t>
+          <t>22-11-2025 04:37</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
@@ -7204,7 +7204,7 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>15115</v>
+        <v>15117</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
@@ -7213,7 +7213,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>22-11-2025 04:15</t>
+          <t>22-11-2025 04:32</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
@@ -7519,7 +7519,7 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>14743</v>
+        <v>14742</v>
       </c>
       <c r="F162" t="inlineStr">
         <is>
@@ -7528,7 +7528,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>21-11-2025 14:54</t>
+          <t>22-11-2025 04:36</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -8006,7 +8006,7 @@
         </is>
       </c>
       <c r="E173" t="n">
-        <v>13543</v>
+        <v>13544</v>
       </c>
       <c r="F173" t="inlineStr">
         <is>
@@ -8015,7 +8015,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>22-11-2025 03:21</t>
+          <t>22-11-2025 04:18</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -8271,7 +8271,7 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>13024</v>
+        <v>13026</v>
       </c>
       <c r="F179" t="inlineStr">
         <is>
@@ -8280,7 +8280,7 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>22-11-2025 04:13</t>
+          <t>22-11-2025 04:34</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
@@ -8527,11 +8527,11 @@
         </is>
       </c>
       <c r="E185" t="n">
-        <v>12246</v>
+        <v>12247</v>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>21-11-2025 14:14</t>
+          <t>22-11-2025 04:31</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
@@ -8923,7 +8923,7 @@
         </is>
       </c>
       <c r="E194" t="n">
-        <v>11510</v>
+        <v>11511</v>
       </c>
       <c r="F194" t="inlineStr">
         <is>
@@ -8932,7 +8932,7 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>22-11-2025 03:33</t>
+          <t>22-11-2025 04:24</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
@@ -9495,7 +9495,7 @@
         </is>
       </c>
       <c r="E207" t="n">
-        <v>9708</v>
+        <v>9709</v>
       </c>
       <c r="F207" t="inlineStr">
         <is>
@@ -9504,7 +9504,7 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>22-11-2025 01:37</t>
+          <t>22-11-2025 04:18</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
@@ -9667,7 +9667,7 @@
         </is>
       </c>
       <c r="E211" t="n">
-        <v>9222</v>
+        <v>9223</v>
       </c>
       <c r="F211" t="inlineStr">
         <is>
@@ -9676,7 +9676,7 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>22-11-2025 02:49</t>
+          <t>22-11-2025 04:33</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
@@ -10408,7 +10408,7 @@
         </is>
       </c>
       <c r="E228" t="n">
-        <v>7989</v>
+        <v>7991</v>
       </c>
       <c r="F228" t="inlineStr">
         <is>
@@ -10417,7 +10417,7 @@
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>22-11-2025 04:14</t>
+          <t>22-11-2025 04:38</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
@@ -10849,7 +10849,7 @@
         </is>
       </c>
       <c r="E238" t="n">
-        <v>6655</v>
+        <v>6656</v>
       </c>
       <c r="F238" t="inlineStr">
         <is>
@@ -10858,7 +10858,7 @@
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>21-11-2025 23:41</t>
+          <t>22-11-2025 04:38</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
@@ -11551,7 +11551,7 @@
         </is>
       </c>
       <c r="E254" t="n">
-        <v>5485</v>
+        <v>5486</v>
       </c>
       <c r="F254" t="inlineStr">
         <is>
@@ -11560,7 +11560,7 @@
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t>22-11-2025 03:51</t>
+          <t>22-11-2025 04:37</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
@@ -11956,7 +11956,7 @@
         </is>
       </c>
       <c r="E263" t="n">
-        <v>4952</v>
+        <v>4953</v>
       </c>
       <c r="F263" t="inlineStr">
         <is>
@@ -11965,7 +11965,7 @@
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>22-11-2025 03:46</t>
+          <t>22-11-2025 04:21</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
@@ -13411,7 +13411,7 @@
         </is>
       </c>
       <c r="E296" t="n">
-        <v>3367</v>
+        <v>3368</v>
       </c>
       <c r="F296" t="inlineStr">
         <is>
@@ -13420,7 +13420,7 @@
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>22-11-2025 03:40</t>
+          <t>22-11-2025 04:31</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
@@ -14078,11 +14078,11 @@
         </is>
       </c>
       <c r="E311" t="n">
-        <v>2981</v>
+        <v>2982</v>
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>22-11-2025 03:55</t>
+          <t>22-11-2025 04:27</t>
         </is>
       </c>
       <c r="H311" t="inlineStr">
@@ -15045,7 +15045,7 @@
         </is>
       </c>
       <c r="E333" t="n">
-        <v>2422</v>
+        <v>2423</v>
       </c>
       <c r="F333" t="inlineStr">
         <is>
@@ -15054,7 +15054,7 @@
       </c>
       <c r="G333" t="inlineStr">
         <is>
-          <t>22-11-2025 03:06</t>
+          <t>22-11-2025 04:29</t>
         </is>
       </c>
       <c r="H333" t="inlineStr">
@@ -16932,7 +16932,7 @@
         </is>
       </c>
       <c r="E376" t="n">
-        <v>1537</v>
+        <v>1538</v>
       </c>
       <c r="F376" t="inlineStr">
         <is>
@@ -16941,7 +16941,7 @@
       </c>
       <c r="G376" t="inlineStr">
         <is>
-          <t>19-11-2025 10:34</t>
+          <t>22-11-2025 04:31</t>
         </is>
       </c>
       <c r="H376" t="inlineStr">
@@ -18593,11 +18593,11 @@
         </is>
       </c>
       <c r="E414" t="n">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="G414" t="inlineStr">
         <is>
-          <t>22-11-2025 02:52</t>
+          <t>22-11-2025 04:20</t>
         </is>
       </c>
       <c r="H414" t="inlineStr">
@@ -19422,7 +19422,7 @@
         </is>
       </c>
       <c r="E433" t="n">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="F433" t="inlineStr">
         <is>
@@ -19431,7 +19431,7 @@
       </c>
       <c r="G433" t="inlineStr">
         <is>
-          <t>22-11-2025 03:23</t>
+          <t>22-11-2025 04:32</t>
         </is>
       </c>
       <c r="H433" t="inlineStr">
@@ -22572,7 +22572,7 @@
       </c>
       <c r="G505" t="inlineStr">
         <is>
-          <t>22-11-2025 04:10</t>
+          <t>22-11-2025 04:25</t>
         </is>
       </c>
       <c r="H505" t="inlineStr">

</xml_diff>

<commit_message>
Regenerate files with Back to Top button included
</commit_message>
<xml_diff>
--- a/starred_repos.xlsx
+++ b/starred_repos.xlsx
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>441456</v>
+        <v>441458</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -521,7 +521,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>22-11-2025 04:44</t>
+          <t>22-11-2025 04:50</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -557,11 +557,11 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>416617</v>
+        <v>416618</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>22-11-2025 04:37</t>
+          <t>22-11-2025 04:51</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>380002</v>
+        <v>380003</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -606,7 +606,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>22-11-2025 04:44</t>
+          <t>22-11-2025 04:45</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>270462</v>
+        <v>270465</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>22-11-2025 04:43</t>
+          <t>22-11-2025 04:50</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>157872</v>
+        <v>157875</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -906,7 +906,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>22-11-2025 04:42</t>
+          <t>22-11-2025 04:49</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>136765</v>
+        <v>136766</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -996,7 +996,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>22-11-2025 04:43</t>
+          <t>22-11-2025 04:47</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1032,7 +1032,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>135877</v>
+        <v>135876</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>22-11-2025 04:39</t>
+          <t>22-11-2025 04:46</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>131401</v>
+        <v>131402</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>22-11-2025 04:42</t>
+          <t>22-11-2025 04:45</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>115895</v>
+        <v>115896</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>22-11-2025 04:20</t>
+          <t>22-11-2025 04:46</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>115456</v>
+        <v>115457</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1387,11 +1387,11 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>101007</v>
+        <v>101008</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>22-11-2025 04:43</t>
+          <t>22-11-2025 04:45</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1602,7 +1602,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>86470</v>
+        <v>86471</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1611,7 +1611,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>22-11-2025 04:01</t>
+          <t>22-11-2025 04:45</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1647,7 +1647,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>84715</v>
+        <v>84717</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>22-11-2025 04:41</t>
+          <t>22-11-2025 04:46</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1692,7 +1692,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>83954</v>
+        <v>83956</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>22-11-2025 04:41</t>
+          <t>22-11-2025 04:46</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1782,11 +1782,11 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>79933</v>
+        <v>79934</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>22-11-2025 03:35</t>
+          <t>22-11-2025 04:47</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1822,7 +1822,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>79376</v>
+        <v>79377</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1831,7 +1831,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>22-11-2025 03:42</t>
+          <t>22-11-2025 04:49</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>75897</v>
+        <v>75898</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>22-11-2025 04:42</t>
+          <t>22-11-2025 04:47</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>22-11-2025 04:32</t>
+          <t>22-11-2025 04:49</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2959,7 +2959,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>47436</v>
+        <v>47437</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -2968,7 +2968,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>22-11-2025 04:41</t>
+          <t>22-11-2025 04:49</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3611,7 +3611,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>37383</v>
+        <v>37384</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>22-11-2025 04:09</t>
+          <t>22-11-2025 04:51</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -9319,7 +9319,7 @@
         </is>
       </c>
       <c r="E203" t="n">
-        <v>9946</v>
+        <v>9947</v>
       </c>
       <c r="F203" t="inlineStr">
         <is>
@@ -9328,7 +9328,7 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>22-11-2025 03:45</t>
+          <t>22-11-2025 04:49</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
@@ -10408,7 +10408,7 @@
         </is>
       </c>
       <c r="E228" t="n">
-        <v>7991</v>
+        <v>7993</v>
       </c>
       <c r="F228" t="inlineStr">
         <is>
@@ -10417,7 +10417,7 @@
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>22-11-2025 04:38</t>
+          <t>22-11-2025 04:49</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
@@ -19422,7 +19422,7 @@
         </is>
       </c>
       <c r="E433" t="n">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="F433" t="inlineStr">
         <is>
@@ -19431,7 +19431,7 @@
       </c>
       <c r="G433" t="inlineStr">
         <is>
-          <t>22-11-2025 04:32</t>
+          <t>22-11-2025 04:47</t>
         </is>
       </c>
       <c r="H433" t="inlineStr">

</xml_diff>

<commit_message>
Fix Back to Top button: increase z-index to 99999, improve visibility
</commit_message>
<xml_diff>
--- a/starred_repos.xlsx
+++ b/starred_repos.xlsx
@@ -557,11 +557,11 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>416618</v>
+        <v>416619</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>22-11-2025 04:51</t>
+          <t>22-11-2025 04:52</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>270465</v>
+        <v>270464</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>22-11-2025 04:50</t>
+          <t>22-11-2025 04:52</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1342,7 +1342,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>102443</v>
+        <v>102442</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>22-11-2025 04:37</t>
+          <t>22-11-2025 04:52</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>93787</v>
+        <v>93788</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>22-11-2025 04:39</t>
+          <t>22-11-2025 04:52</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1647,7 +1647,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>84717</v>
+        <v>84718</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>22-11-2025 04:46</t>
+          <t>22-11-2025 04:52</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1692,7 +1692,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>83956</v>
+        <v>83957</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>22-11-2025 04:46</t>
+          <t>22-11-2025 04:52</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1822,7 +1822,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>79377</v>
+        <v>79378</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1831,7 +1831,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>22-11-2025 04:49</t>
+          <t>22-11-2025 04:52</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>56211</v>
+        <v>56212</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>22-11-2025 03:33</t>
+          <t>22-11-2025 04:52</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2433,7 +2433,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>53639</v>
+        <v>53640</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>22-11-2025 04:16</t>
+          <t>22-11-2025 04:52</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3129,7 +3129,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>43209</v>
+        <v>43211</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>22-11-2025 04:20</t>
+          <t>22-11-2025 04:52</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -5530,7 +5530,7 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>22127</v>
+        <v>22128</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -5539,7 +5539,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>22-11-2025 04:35</t>
+          <t>22-11-2025 04:52</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -6767,7 +6767,7 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>16330</v>
+        <v>16331</v>
       </c>
       <c r="F145" t="inlineStr">
         <is>
@@ -6776,7 +6776,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>22-11-2025 04:19</t>
+          <t>22-11-2025 04:52</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
@@ -12001,11 +12001,11 @@
         </is>
       </c>
       <c r="E264" t="n">
-        <v>4948</v>
+        <v>4949</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>22-11-2025 04:01</t>
+          <t>22-11-2025 04:52</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
@@ -14082,7 +14082,7 @@
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>22-11-2025 04:43</t>
+          <t>22-11-2025 04:52</t>
         </is>
       </c>
       <c r="H311" t="inlineStr">

</xml_diff>

<commit_message>
Make Back to Top button always visible
</commit_message>
<xml_diff>
--- a/starred_repos.xlsx
+++ b/starred_repos.xlsx
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>441460</v>
+        <v>441462</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -521,7 +521,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>22-11-2025 04:56</t>
+          <t>22-11-2025 05:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>270466</v>
+        <v>270468</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>22-11-2025 04:55</t>
+          <t>22-11-2025 05:01</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -687,11 +687,11 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>259315</v>
+        <v>259316</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>22-11-2025 04:55</t>
+          <t>22-11-2025 04:57</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -727,11 +727,11 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>250560</v>
+        <v>250561</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>22-11-2025 04:37</t>
+          <t>22-11-2025 05:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>198029</v>
+        <v>198030</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -776,7 +776,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>22-11-2025 04:38</t>
+          <t>22-11-2025 04:57</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>131402</v>
+        <v>131403</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>22-11-2025 04:45</t>
+          <t>22-11-2025 04:56</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>56212</v>
+        <v>56213</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>22-11-2025 04:52</t>
+          <t>22-11-2025 04:57</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2698,7 +2698,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>51325</v>
+        <v>51326</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>22-11-2025 04:26</t>
+          <t>22-11-2025 04:59</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3093,7 +3093,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>22-11-2025 04:41</t>
+          <t>22-11-2025 04:59</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -3129,7 +3129,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>43211</v>
+        <v>43212</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>22-11-2025 04:52</t>
+          <t>22-11-2025 04:57</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -5616,7 +5616,7 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>21908</v>
+        <v>21909</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
@@ -5625,7 +5625,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>22-11-2025 03:22</t>
+          <t>22-11-2025 04:58</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -6142,7 +6142,7 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>18612</v>
+        <v>18613</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -6151,7 +6151,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>22-11-2025 04:54</t>
+          <t>22-11-2025 04:58</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -8271,7 +8271,7 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>13028</v>
+        <v>13029</v>
       </c>
       <c r="F179" t="inlineStr">
         <is>
@@ -8280,7 +8280,7 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>22-11-2025 04:43</t>
+          <t>22-11-2025 04:58</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
@@ -9431,67 +9431,63 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>bytebot-ai/bytebot</t>
+          <t>BeehiveInnovations/zen-mcp-server</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>https://github.com/bytebot-ai/bytebot</t>
+          <t>https://github.com/BeehiveInnovations/zen-mcp-server</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>AI/ML</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Bytebot is a self-hosted AI desktop agent that automates computer tasks through natural language commands, operating within a containerized Linux desktop environment.</t>
+          <t>The power of Claude Code / GeminiCLI / CodexCLI + [Gemini / OpenAI / OpenRouter / Azure / Grok / Ollama / Custom Model / All Of The Above] working as one.</t>
         </is>
       </c>
       <c r="E206" t="n">
-        <v>9709</v>
+        <v>9710</v>
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>22-11-2025 04:15</t>
+          <t>22-11-2025 04:58</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>03-02-2025 18:18</t>
-        </is>
-      </c>
-      <c r="I206" t="inlineStr">
-        <is>
-          <t>agent, agentic-ai, agents, ai, ai-agents</t>
-        </is>
-      </c>
+          <t>08-06-2025 15:36</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>BeehiveInnovations/zen-mcp-server</t>
+          <t>bytebot-ai/bytebot</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>https://github.com/BeehiveInnovations/zen-mcp-server</t>
+          <t>https://github.com/bytebot-ai/bytebot</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>AI/ML</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>The power of Claude Code / GeminiCLI / CodexCLI + [Gemini / OpenAI / OpenRouter / Azure / Grok / Ollama / Custom Model / All Of The Above] working as one.</t>
+          <t>Bytebot is a self-hosted AI desktop agent that automates computer tasks through natural language commands, operating within a containerized Linux desktop environment.</t>
         </is>
       </c>
       <c r="E207" t="n">
@@ -9499,20 +9495,24 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>22-11-2025 04:18</t>
+          <t>22-11-2025 04:15</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>08-06-2025 15:36</t>
-        </is>
-      </c>
-      <c r="I207" t="inlineStr"/>
+          <t>03-02-2025 18:18</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>agent, agentic-ai, agents, ai, ai-agents</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -10628,7 +10628,7 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>7405</v>
+        <v>7406</v>
       </c>
       <c r="F233" t="inlineStr">
         <is>
@@ -10637,7 +10637,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>22-11-2025 03:31</t>
+          <t>22-11-2025 04:57</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
@@ -13195,7 +13195,7 @@
         </is>
       </c>
       <c r="E291" t="n">
-        <v>3635</v>
+        <v>3636</v>
       </c>
       <c r="F291" t="inlineStr">
         <is>
@@ -13204,7 +13204,7 @@
       </c>
       <c r="G291" t="inlineStr">
         <is>
-          <t>22-11-2025 03:33</t>
+          <t>22-11-2025 04:57</t>
         </is>
       </c>
       <c r="H291" t="inlineStr">
@@ -14910,7 +14910,7 @@
         </is>
       </c>
       <c r="E330" t="n">
-        <v>2560</v>
+        <v>2561</v>
       </c>
       <c r="F330" t="inlineStr">
         <is>
@@ -14919,7 +14919,7 @@
       </c>
       <c r="G330" t="inlineStr">
         <is>
-          <t>22-11-2025 03:31</t>
+          <t>22-11-2025 04:57</t>
         </is>
       </c>
       <c r="H330" t="inlineStr">

</xml_diff>

<commit_message>
Fix Back to Top button: add onclick handler, elegant SVG chevron icon, circular design
</commit_message>
<xml_diff>
--- a/starred_repos.xlsx
+++ b/starred_repos.xlsx
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>441462</v>
+        <v>441464</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -521,7 +521,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>22-11-2025 05:00</t>
+          <t>22-11-2025 05:07</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -557,11 +557,11 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>416621</v>
+        <v>416625</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>22-11-2025 04:55</t>
+          <t>22-11-2025 05:10</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>270468</v>
+        <v>270473</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>22-11-2025 05:01</t>
+          <t>22-11-2025 05:12</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -687,11 +687,11 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>259316</v>
+        <v>259317</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>22-11-2025 04:57</t>
+          <t>22-11-2025 05:02</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -727,11 +727,11 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>250561</v>
+        <v>250562</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>22-11-2025 05:00</t>
+          <t>22-11-2025 05:04</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -812,11 +812,11 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>195126</v>
+        <v>195127</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>22-11-2025 04:56</t>
+          <t>22-11-2025 05:08</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>157875</v>
+        <v>157876</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -906,7 +906,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>22-11-2025 04:49</t>
+          <t>22-11-2025 05:08</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>157019</v>
+        <v>157021</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -951,7 +951,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>22-11-2025 04:33</t>
+          <t>22-11-2025 05:11</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>22-11-2025 04:47</t>
+          <t>22-11-2025 05:07</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1032,7 +1032,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>135876</v>
+        <v>135877</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>22-11-2025 04:46</t>
+          <t>22-11-2025 05:05</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1122,7 +1122,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>125896</v>
+        <v>125897</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>22-11-2025 03:49</t>
+          <t>22-11-2025 05:12</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>115896</v>
+        <v>115897</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>22-11-2025 04:46</t>
+          <t>22-11-2025 05:10</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>115458</v>
+        <v>115463</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>22-11-2025 04:55</t>
+          <t>22-11-2025 05:11</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>22-11-2025 04:52</t>
+          <t>22-11-2025 05:08</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1647,7 +1647,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>84718</v>
+        <v>84719</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>22-11-2025 04:52</t>
+          <t>22-11-2025 05:01</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1822,7 +1822,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>79378</v>
+        <v>79379</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1831,7 +1831,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>22-11-2025 04:52</t>
+          <t>22-11-2025 05:09</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>68291</v>
+        <v>68290</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2056,7 +2056,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>22-11-2025 04:49</t>
+          <t>22-11-2025 05:05</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>22-11-2025 04:56</t>
+          <t>22-11-2025 05:09</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>56213</v>
+        <v>56214</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>22-11-2025 04:57</t>
+          <t>22-11-2025 05:03</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3170,7 +3170,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>43134</v>
+        <v>43135</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -3179,7 +3179,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>22-11-2025 04:21</t>
+          <t>22-11-2025 05:07</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3341,7 +3341,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>39416</v>
+        <v>39417</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -3350,7 +3350,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>22-11-2025 03:08</t>
+          <t>22-11-2025 05:11</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3386,7 +3386,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>39214</v>
+        <v>39215</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -3395,7 +3395,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>22-11-2025 03:31</t>
+          <t>22-11-2025 05:01</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3746,7 +3746,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>35658</v>
+        <v>35657</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -3755,7 +3755,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>22-11-2025 04:17</t>
+          <t>22-11-2025 05:12</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -4442,7 +4442,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>28897</v>
+        <v>28898</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>22-11-2025 01:40</t>
+          <t>22-11-2025 05:08</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -6502,7 +6502,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>17445</v>
+        <v>17446</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
@@ -6511,7 +6511,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>22-11-2025 04:44</t>
+          <t>22-11-2025 05:11</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -7073,7 +7073,7 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>15663</v>
+        <v>15664</v>
       </c>
       <c r="F152" t="inlineStr">
         <is>
@@ -7082,7 +7082,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>22-11-2025 04:37</t>
+          <t>22-11-2025 05:03</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
@@ -7204,7 +7204,7 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>15118</v>
+        <v>15123</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
@@ -7213,7 +7213,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>22-11-2025 04:39</t>
+          <t>22-11-2025 05:12</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
@@ -7564,7 +7564,7 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>14676</v>
+        <v>14677</v>
       </c>
       <c r="F163" t="inlineStr">
         <is>
@@ -7573,7 +7573,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>22-11-2025 01:33</t>
+          <t>22-11-2025 05:09</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
@@ -8006,7 +8006,7 @@
         </is>
       </c>
       <c r="E173" t="n">
-        <v>13545</v>
+        <v>13546</v>
       </c>
       <c r="F173" t="inlineStr">
         <is>
@@ -8015,7 +8015,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>22-11-2025 04:52</t>
+          <t>22-11-2025 05:10</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -8316,11 +8316,11 @@
         </is>
       </c>
       <c r="E180" t="n">
-        <v>12872</v>
+        <v>12873</v>
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>21-11-2025 21:42</t>
+          <t>22-11-2025 05:03</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
@@ -9319,7 +9319,7 @@
         </is>
       </c>
       <c r="E203" t="n">
-        <v>9947</v>
+        <v>9948</v>
       </c>
       <c r="F203" t="inlineStr">
         <is>
@@ -9328,7 +9328,7 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>22-11-2025 04:49</t>
+          <t>22-11-2025 05:09</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
@@ -9802,11 +9802,11 @@
         </is>
       </c>
       <c r="E214" t="n">
-        <v>8978</v>
+        <v>8979</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>22-11-2025 04:14</t>
+          <t>22-11-2025 05:05</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
@@ -10156,7 +10156,7 @@
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>21-11-2025 23:31</t>
+          <t>22-11-2025 05:01</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
@@ -10628,7 +10628,7 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>7406</v>
+        <v>7407</v>
       </c>
       <c r="F233" t="inlineStr">
         <is>
@@ -10637,7 +10637,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>22-11-2025 04:57</t>
+          <t>22-11-2025 05:01</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
@@ -13195,7 +13195,7 @@
         </is>
       </c>
       <c r="E291" t="n">
-        <v>3636</v>
+        <v>3637</v>
       </c>
       <c r="F291" t="inlineStr">
         <is>
@@ -13204,7 +13204,7 @@
       </c>
       <c r="G291" t="inlineStr">
         <is>
-          <t>22-11-2025 04:57</t>
+          <t>22-11-2025 05:01</t>
         </is>
       </c>
       <c r="H291" t="inlineStr">
@@ -13501,7 +13501,7 @@
         </is>
       </c>
       <c r="E298" t="n">
-        <v>3249</v>
+        <v>3250</v>
       </c>
       <c r="F298" t="inlineStr">
         <is>
@@ -13510,7 +13510,7 @@
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>22-11-2025 03:57</t>
+          <t>22-11-2025 05:03</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">
@@ -13771,7 +13771,7 @@
         </is>
       </c>
       <c r="E304" t="n">
-        <v>3146</v>
+        <v>3147</v>
       </c>
       <c r="F304" t="inlineStr">
         <is>
@@ -13780,7 +13780,7 @@
       </c>
       <c r="G304" t="inlineStr">
         <is>
-          <t>21-11-2025 23:17</t>
+          <t>22-11-2025 05:12</t>
         </is>
       </c>
       <c r="H304" t="inlineStr">
@@ -14253,7 +14253,7 @@
         </is>
       </c>
       <c r="E315" t="n">
-        <v>2953</v>
+        <v>2954</v>
       </c>
       <c r="F315" t="inlineStr">
         <is>
@@ -14262,7 +14262,7 @@
       </c>
       <c r="G315" t="inlineStr">
         <is>
-          <t>21-11-2025 22:55</t>
+          <t>22-11-2025 05:10</t>
         </is>
       </c>
       <c r="H315" t="inlineStr">
@@ -14910,7 +14910,7 @@
         </is>
       </c>
       <c r="E330" t="n">
-        <v>2561</v>
+        <v>2562</v>
       </c>
       <c r="F330" t="inlineStr">
         <is>
@@ -14919,7 +14919,7 @@
       </c>
       <c r="G330" t="inlineStr">
         <is>
-          <t>22-11-2025 04:57</t>
+          <t>22-11-2025 05:01</t>
         </is>
       </c>
       <c r="H330" t="inlineStr">
@@ -16271,7 +16271,7 @@
         </is>
       </c>
       <c r="E361" t="n">
-        <v>1734</v>
+        <v>1735</v>
       </c>
       <c r="F361" t="inlineStr">
         <is>
@@ -16280,7 +16280,7 @@
       </c>
       <c r="G361" t="inlineStr">
         <is>
-          <t>21-11-2025 21:14</t>
+          <t>22-11-2025 05:01</t>
         </is>
       </c>
       <c r="H361" t="inlineStr">
@@ -18516,7 +18516,7 @@
       </c>
       <c r="G412" t="inlineStr">
         <is>
-          <t>22-11-2025 01:47</t>
+          <t>22-11-2025 05:04</t>
         </is>
       </c>
       <c r="H412" t="inlineStr">
@@ -20385,7 +20385,7 @@
         </is>
       </c>
       <c r="E455" t="n">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="F455" t="inlineStr">
         <is>
@@ -20394,7 +20394,7 @@
       </c>
       <c r="G455" t="inlineStr">
         <is>
-          <t>21-11-2025 18:01</t>
+          <t>22-11-2025 05:10</t>
         </is>
       </c>
       <c r="H455" t="inlineStr">
@@ -20822,7 +20822,7 @@
         </is>
       </c>
       <c r="E465" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F465" t="inlineStr">
         <is>
@@ -20831,7 +20831,7 @@
       </c>
       <c r="G465" t="inlineStr">
         <is>
-          <t>21-11-2025 21:10</t>
+          <t>22-11-2025 05:05</t>
         </is>
       </c>
       <c r="H465" t="inlineStr">
@@ -22572,7 +22572,7 @@
       </c>
       <c r="G505" t="inlineStr">
         <is>
-          <t>22-11-2025 04:55</t>
+          <t>22-11-2025 05:11</t>
         </is>
       </c>
       <c r="H505" t="inlineStr">

</xml_diff>

<commit_message>
Fix Back to Top button: correct JavaScript syntax (single braces)
</commit_message>
<xml_diff>
--- a/starred_repos.xlsx
+++ b/starred_repos.xlsx
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>441464</v>
+        <v>441471</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -521,7 +521,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>22-11-2025 05:07</t>
+          <t>22-11-2025 05:28</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -557,11 +557,11 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>416625</v>
+        <v>416626</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>22-11-2025 05:10</t>
+          <t>22-11-2025 05:16</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>380005</v>
+        <v>380007</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -606,7 +606,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>22-11-2025 04:55</t>
+          <t>22-11-2025 05:21</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,11 +687,11 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>259317</v>
+        <v>259319</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>22-11-2025 05:02</t>
+          <t>22-11-2025 05:25</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>198030</v>
+        <v>198029</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -776,7 +776,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>22-11-2025 04:57</t>
+          <t>22-11-2025 05:20</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -812,11 +812,11 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>195127</v>
+        <v>195128</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>22-11-2025 05:08</t>
+          <t>22-11-2025 05:17</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>157876</v>
+        <v>157877</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -906,7 +906,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>22-11-2025 05:08</t>
+          <t>22-11-2025 05:27</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1032,7 +1032,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>135877</v>
+        <v>135878</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>22-11-2025 05:05</t>
+          <t>22-11-2025 05:21</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>115463</v>
+        <v>115465</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>22-11-2025 05:11</t>
+          <t>22-11-2025 05:24</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1297,7 +1297,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>102871</v>
+        <v>102872</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1306,7 +1306,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>22-11-2025 04:36</t>
+          <t>22-11-2025 05:26</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1342,7 +1342,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>102443</v>
+        <v>102444</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>22-11-2025 05:08</t>
+          <t>22-11-2025 05:23</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1387,11 +1387,11 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>101008</v>
+        <v>101010</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>22-11-2025 04:45</t>
+          <t>22-11-2025 05:25</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>93788</v>
+        <v>93789</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>22-11-2025 04:52</t>
+          <t>22-11-2025 05:25</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1562,11 +1562,11 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>88187</v>
+        <v>88188</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>22-11-2025 04:38</t>
+          <t>22-11-2025 05:20</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1692,7 +1692,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>83958</v>
+        <v>83960</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>22-11-2025 04:53</t>
+          <t>22-11-2025 05:23</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1782,11 +1782,11 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>79934</v>
+        <v>79935</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>22-11-2025 04:47</t>
+          <t>22-11-2025 05:26</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>22-11-2025 05:09</t>
+          <t>22-11-2025 05:22</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>56214</v>
+        <v>56215</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>22-11-2025 05:03</t>
+          <t>22-11-2025 05:18</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2433,7 +2433,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>53640</v>
+        <v>53641</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>22-11-2025 04:52</t>
+          <t>22-11-2025 05:28</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2788,7 +2788,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>47892</v>
+        <v>47893</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>22-11-2025 04:23</t>
+          <t>22-11-2025 05:13</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2959,7 +2959,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>47437</v>
+        <v>47441</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -2968,7 +2968,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>22-11-2025 04:49</t>
+          <t>22-11-2025 05:23</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3129,7 +3129,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>43212</v>
+        <v>43217</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>22-11-2025 04:57</t>
+          <t>22-11-2025 05:27</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3170,7 +3170,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>43135</v>
+        <v>43137</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -3179,7 +3179,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>22-11-2025 05:07</t>
+          <t>22-11-2025 05:28</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3215,7 +3215,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>42969</v>
+        <v>42970</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -3224,7 +3224,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>22-11-2025 04:22</t>
+          <t>22-11-2025 05:14</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3611,7 +3611,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>37384</v>
+        <v>37385</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>22-11-2025 04:51</t>
+          <t>22-11-2025 05:17</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3656,7 +3656,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>36935</v>
+        <v>36936</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>22-11-2025 04:26</t>
+          <t>22-11-2025 05:27</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3746,7 +3746,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>35657</v>
+        <v>35658</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -3755,7 +3755,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>22-11-2025 05:12</t>
+          <t>22-11-2025 05:27</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -3791,7 +3791,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>35499</v>
+        <v>35500</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -3800,7 +3800,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>22-11-2025 02:40</t>
+          <t>22-11-2025 05:24</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -3876,7 +3876,7 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>34502</v>
+        <v>34503</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>22-11-2025 04:41</t>
+          <t>22-11-2025 05:21</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -4092,7 +4092,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>31853</v>
+        <v>31854</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -4101,7 +4101,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>22-11-2025 04:36</t>
+          <t>22-11-2025 05:19</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -4262,7 +4262,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>31442</v>
+        <v>31443</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -4271,7 +4271,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>22-11-2025 04:32</t>
+          <t>22-11-2025 05:14</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -4352,7 +4352,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>29826</v>
+        <v>29827</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -4361,7 +4361,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>22-11-2025 04:35</t>
+          <t>22-11-2025 05:19</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -4442,7 +4442,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>28898</v>
+        <v>28900</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>22-11-2025 05:08</t>
+          <t>22-11-2025 05:17</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -4747,7 +4747,7 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>26860</v>
+        <v>26861</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -4756,7 +4756,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>22-11-2025 04:35</t>
+          <t>22-11-2025 05:19</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -4837,7 +4837,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>26089</v>
+        <v>26090</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -4846,7 +4846,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>22-11-2025 00:31</t>
+          <t>22-11-2025 05:28</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -5139,7 +5139,7 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>25056</v>
+        <v>25057</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>21-11-2025 23:10</t>
+          <t>22-11-2025 05:21</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -5404,7 +5404,7 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>23142</v>
+        <v>23143</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
@@ -5413,7 +5413,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>22-11-2025 02:02</t>
+          <t>22-11-2025 05:17</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -5489,7 +5489,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>22315</v>
+        <v>22316</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>22-11-2025 04:53</t>
+          <t>22-11-2025 05:25</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -6142,7 +6142,7 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>18613</v>
+        <v>18612</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -6151,7 +6151,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>22-11-2025 04:58</t>
+          <t>22-11-2025 05:22</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -6592,7 +6592,7 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>17277</v>
+        <v>17278</v>
       </c>
       <c r="F141" t="inlineStr">
         <is>
@@ -6601,7 +6601,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>22-11-2025 04:11</t>
+          <t>22-11-2025 05:14</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -6767,7 +6767,7 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>16331</v>
+        <v>16332</v>
       </c>
       <c r="F145" t="inlineStr">
         <is>
@@ -6776,7 +6776,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>22-11-2025 04:52</t>
+          <t>22-11-2025 05:15</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
@@ -7073,7 +7073,7 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>15664</v>
+        <v>15666</v>
       </c>
       <c r="F152" t="inlineStr">
         <is>
@@ -7082,7 +7082,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>22-11-2025 05:03</t>
+          <t>22-11-2025 05:21</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
@@ -7204,7 +7204,7 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>15123</v>
+        <v>15124</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
@@ -7213,7 +7213,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>22-11-2025 05:12</t>
+          <t>22-11-2025 05:28</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
@@ -7294,7 +7294,7 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>15040</v>
+        <v>15041</v>
       </c>
       <c r="F157" t="inlineStr">
         <is>
@@ -7303,7 +7303,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>22-11-2025 03:21</t>
+          <t>22-11-2025 05:23</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -7384,7 +7384,7 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>14864</v>
+        <v>14865</v>
       </c>
       <c r="F159" t="inlineStr">
         <is>
@@ -7393,7 +7393,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>22-11-2025 01:19</t>
+          <t>22-11-2025 05:21</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
@@ -7916,7 +7916,7 @@
         </is>
       </c>
       <c r="E171" t="n">
-        <v>13738</v>
+        <v>13739</v>
       </c>
       <c r="F171" t="inlineStr">
         <is>
@@ -7925,7 +7925,7 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>22-11-2025 03:43</t>
+          <t>22-11-2025 05:22</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
@@ -8181,7 +8181,7 @@
         </is>
       </c>
       <c r="E177" t="n">
-        <v>13180</v>
+        <v>13181</v>
       </c>
       <c r="F177" t="inlineStr">
         <is>
@@ -8190,7 +8190,7 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>22-11-2025 00:39</t>
+          <t>22-11-2025 05:23</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
@@ -8271,7 +8271,7 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>13029</v>
+        <v>13031</v>
       </c>
       <c r="F179" t="inlineStr">
         <is>
@@ -8280,7 +8280,7 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>22-11-2025 04:58</t>
+          <t>22-11-2025 05:19</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
@@ -8563,7 +8563,7 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>12225</v>
+        <v>12226</v>
       </c>
       <c r="F186" t="inlineStr">
         <is>
@@ -8572,7 +8572,7 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>22-11-2025 00:45</t>
+          <t>22-11-2025 05:24</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
@@ -9431,22 +9431,22 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>BeehiveInnovations/zen-mcp-server</t>
+          <t>bytebot-ai/bytebot</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>https://github.com/BeehiveInnovations/zen-mcp-server</t>
+          <t>https://github.com/bytebot-ai/bytebot</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>AI/ML</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>The power of Claude Code / GeminiCLI / CodexCLI + [Gemini / OpenAI / OpenRouter / Azure / Grok / Ollama / Custom Model / All Of The Above] working as one.</t>
+          <t>Bytebot is a self-hosted AI desktop agent that automates computer tasks through natural language commands, operating within a containerized Linux desktop environment.</t>
         </is>
       </c>
       <c r="E206" t="n">
@@ -9454,65 +9454,65 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>22-11-2025 04:58</t>
+          <t>22-11-2025 05:16</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>08-06-2025 15:36</t>
-        </is>
-      </c>
-      <c r="I206" t="inlineStr"/>
+          <t>03-02-2025 18:18</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>agent, agentic-ai, agents, ai, ai-agents</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>bytebot-ai/bytebot</t>
+          <t>BeehiveInnovations/zen-mcp-server</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>https://github.com/bytebot-ai/bytebot</t>
+          <t>https://github.com/BeehiveInnovations/zen-mcp-server</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>AI/ML</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Bytebot is a self-hosted AI desktop agent that automates computer tasks through natural language commands, operating within a containerized Linux desktop environment.</t>
+          <t>The power of Claude Code / GeminiCLI / CodexCLI + [Gemini / OpenAI / OpenRouter / Azure / Grok / Ollama / Custom Model / All Of The Above] working as one.</t>
         </is>
       </c>
       <c r="E207" t="n">
-        <v>9709</v>
+        <v>9710</v>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>22-11-2025 04:15</t>
+          <t>22-11-2025 04:58</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>03-02-2025 18:18</t>
-        </is>
-      </c>
-      <c r="I207" t="inlineStr">
-        <is>
-          <t>agent, agentic-ai, agents, ai, ai-agents</t>
-        </is>
-      </c>
+          <t>08-06-2025 15:36</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -9712,7 +9712,7 @@
         </is>
       </c>
       <c r="E212" t="n">
-        <v>9127</v>
+        <v>9128</v>
       </c>
       <c r="F212" t="inlineStr">
         <is>
@@ -9721,7 +9721,7 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>22-11-2025 02:49</t>
+          <t>22-11-2025 05:16</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
@@ -9927,7 +9927,7 @@
         </is>
       </c>
       <c r="E217" t="n">
-        <v>8672</v>
+        <v>8673</v>
       </c>
       <c r="F217" t="inlineStr">
         <is>
@@ -9936,7 +9936,7 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>22-11-2025 00:21</t>
+          <t>22-11-2025 05:17</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
@@ -11286,7 +11286,7 @@
         </is>
       </c>
       <c r="E248" t="n">
-        <v>6101</v>
+        <v>6102</v>
       </c>
       <c r="F248" t="inlineStr">
         <is>
@@ -11295,7 +11295,7 @@
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>21-11-2025 14:00</t>
+          <t>22-11-2025 05:20</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
@@ -11821,7 +11821,7 @@
         </is>
       </c>
       <c r="E260" t="n">
-        <v>5082</v>
+        <v>5083</v>
       </c>
       <c r="F260" t="inlineStr">
         <is>
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>21-11-2025 22:10</t>
+          <t>22-11-2025 05:26</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
@@ -12266,7 +12266,7 @@
         </is>
       </c>
       <c r="E270" t="n">
-        <v>4712</v>
+        <v>4713</v>
       </c>
       <c r="F270" t="inlineStr">
         <is>
@@ -12275,7 +12275,7 @@
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>21-11-2025 16:24</t>
+          <t>22-11-2025 05:27</t>
         </is>
       </c>
       <c r="H270" t="inlineStr">
@@ -13501,7 +13501,7 @@
         </is>
       </c>
       <c r="E298" t="n">
-        <v>3250</v>
+        <v>3251</v>
       </c>
       <c r="F298" t="inlineStr">
         <is>
@@ -13510,7 +13510,7 @@
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>22-11-2025 05:03</t>
+          <t>22-11-2025 05:14</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">
@@ -13861,7 +13861,7 @@
         </is>
       </c>
       <c r="E306" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="F306" t="inlineStr">
         <is>
@@ -13870,7 +13870,7 @@
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t>21-11-2025 22:42</t>
+          <t>22-11-2025 05:28</t>
         </is>
       </c>
       <c r="H306" t="inlineStr">
@@ -14082,7 +14082,7 @@
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>22-11-2025 04:52</t>
+          <t>22-11-2025 05:22</t>
         </is>
       </c>
       <c r="H311" t="inlineStr">
@@ -14429,11 +14429,11 @@
         </is>
       </c>
       <c r="E319" t="n">
-        <v>2824</v>
+        <v>2825</v>
       </c>
       <c r="G319" t="inlineStr">
         <is>
-          <t>22-11-2025 03:56</t>
+          <t>22-11-2025 05:18</t>
         </is>
       </c>
       <c r="H319" t="inlineStr">
@@ -15045,7 +15045,7 @@
         </is>
       </c>
       <c r="E333" t="n">
-        <v>2423</v>
+        <v>2424</v>
       </c>
       <c r="F333" t="inlineStr">
         <is>
@@ -15054,7 +15054,7 @@
       </c>
       <c r="G333" t="inlineStr">
         <is>
-          <t>22-11-2025 04:29</t>
+          <t>22-11-2025 05:16</t>
         </is>
       </c>
       <c r="H333" t="inlineStr">
@@ -15126,7 +15126,7 @@
         </is>
       </c>
       <c r="E335" t="n">
-        <v>2340</v>
+        <v>2341</v>
       </c>
       <c r="F335" t="inlineStr">
         <is>
@@ -15135,7 +15135,7 @@
       </c>
       <c r="G335" t="inlineStr">
         <is>
-          <t>22-11-2025 01:58</t>
+          <t>22-11-2025 05:15</t>
         </is>
       </c>
       <c r="H335" t="inlineStr">
@@ -19358,90 +19358,90 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>LLM-Red-Team/glm-free-api</t>
+          <t>raghavyuva/nixopus</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>https://github.com/LLM-Red-Team/glm-free-api</t>
+          <t>https://github.com/raghavyuva/nixopus</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>AI/ML</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>🚀 智谱清言ChatGLM-4-Plus大模型逆向API【特长：超强智能体】，支持高速流式输出、支持智能体对话、支持多轮对话、支持沉思模型、支持Zero思考推理模型、支持视频生成、支持AI绘图、支持联网搜索、支持长文档解读、支持代码调用、支持图像解析，零配置部署，多路token支持，自动清理会话痕迹，仅供测试，如需商用请前往官方开放平台。</t>
+          <t>Open Source Alternative to vercel, heroku, netlify with simplified workflows</t>
         </is>
       </c>
       <c r="E432" t="n">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="F432" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>Go</t>
         </is>
       </c>
       <c r="G432" t="inlineStr">
         <is>
-          <t>20-11-2025 15:00</t>
+          <t>22-11-2025 05:25</t>
         </is>
       </c>
       <c r="H432" t="inlineStr">
         <is>
-          <t>17-03-2024 07:53</t>
+          <t>21-02-2025 11:17</t>
         </is>
       </c>
       <c r="I432" t="inlineStr">
         <is>
-          <t>chat-api, chatbot, chatglm-4, chatglm-api, deepresearch</t>
+          <t>ci-cd, coolify, deployment, file-manager, golang</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>raghavyuva/nixopus</t>
+          <t>LLM-Red-Team/glm-free-api</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>https://github.com/raghavyuva/nixopus</t>
+          <t>https://github.com/LLM-Red-Team/glm-free-api</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>DevOps</t>
+          <t>AI/ML</t>
         </is>
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>Open Source Alternative to vercel, heroku, netlify with simplified workflows</t>
+          <t>🚀 智谱清言ChatGLM-4-Plus大模型逆向API【特长：超强智能体】，支持高速流式输出、支持智能体对话、支持多轮对话、支持沉思模型、支持Zero思考推理模型、支持视频生成、支持AI绘图、支持联网搜索、支持长文档解读、支持代码调用、支持图像解析，零配置部署，多路token支持，自动清理会话痕迹，仅供测试，如需商用请前往官方开放平台。</t>
         </is>
       </c>
       <c r="E433" t="n">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="F433" t="inlineStr">
         <is>
-          <t>Go</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G433" t="inlineStr">
         <is>
-          <t>22-11-2025 04:54</t>
+          <t>20-11-2025 15:00</t>
         </is>
       </c>
       <c r="H433" t="inlineStr">
         <is>
-          <t>21-02-2025 11:17</t>
+          <t>17-03-2024 07:53</t>
         </is>
       </c>
       <c r="I433" t="inlineStr">
         <is>
-          <t>ci-cd, coolify, deployment, file-manager, golang</t>
+          <t>chat-api, chatbot, chatglm-4, chatglm-api, deepresearch</t>
         </is>
       </c>
     </row>
@@ -19737,7 +19737,7 @@
       </c>
       <c r="G440" t="inlineStr">
         <is>
-          <t>22-11-2025 02:20</t>
+          <t>22-11-2025 05:16</t>
         </is>
       </c>
       <c r="H440" t="inlineStr">
@@ -22572,7 +22572,7 @@
       </c>
       <c r="G505" t="inlineStr">
         <is>
-          <t>22-11-2025 05:11</t>
+          <t>22-11-2025 05:26</t>
         </is>
       </c>
       <c r="H505" t="inlineStr">

</xml_diff>